<commit_message>
line chart added for lipfendra and table dynamic
</commit_message>
<xml_diff>
--- a/NAP mock data.xlsx
+++ b/NAP mock data.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A585BCF-510A-4B2C-A6C4-94E29E038496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC561869-D2D5-4A1D-824E-BD4C11E46DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Market growth" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="327">
   <si>
     <t>Year</t>
   </si>
@@ -1095,7 +1095,7 @@
     <numFmt numFmtId="167" formatCode="0.00&quot;M&quot;"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1199,6 +1199,14 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="14">
@@ -1573,7 +1581,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1794,17 +1802,26 @@
     </xf>
     <xf numFmtId="3" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3799,6 +3816,8 @@
     <col min="4" max="4" width="20.109375" customWidth="1"/>
     <col min="5" max="5" width="22.5546875" customWidth="1"/>
     <col min="6" max="6" width="16.109375" customWidth="1"/>
+    <col min="8" max="8" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.21875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:13" ht="46.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -4048,8 +4067,12 @@
         <v>128</v>
       </c>
       <c r="G13" s="52"/>
-      <c r="H13" s="52"/>
-      <c r="I13" s="52"/>
+      <c r="H13" s="93" t="s">
+        <v>58</v>
+      </c>
+      <c r="I13" s="93" t="s">
+        <v>128</v>
+      </c>
     </row>
     <row r="14" spans="2:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B14" s="63">
@@ -4068,8 +4091,12 @@
         <v>131</v>
       </c>
       <c r="G14" s="58"/>
-      <c r="H14" s="58"/>
-      <c r="I14" s="58"/>
+      <c r="H14" s="94">
+        <v>46204</v>
+      </c>
+      <c r="I14" s="92" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="15" spans="2:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B15" s="63">
@@ -4088,8 +4115,12 @@
         <v>133</v>
       </c>
       <c r="G15" s="58"/>
-      <c r="H15" s="58"/>
-      <c r="I15" s="58"/>
+      <c r="H15" s="94">
+        <v>46235</v>
+      </c>
+      <c r="I15" s="92" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="16" spans="2:13" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B16" s="63">
@@ -4108,8 +4139,12 @@
         <v>135</v>
       </c>
       <c r="G16" s="58"/>
-      <c r="H16" s="58"/>
-      <c r="I16" s="58"/>
+      <c r="H16" s="94">
+        <v>46266</v>
+      </c>
+      <c r="I16" s="92" t="s">
+        <v>135</v>
+      </c>
     </row>
     <row r="17" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B17" s="63">
@@ -4128,8 +4163,12 @@
         <v>137</v>
       </c>
       <c r="G17" s="58"/>
-      <c r="H17" s="58"/>
-      <c r="I17" s="58"/>
+      <c r="H17" s="94">
+        <v>46296</v>
+      </c>
+      <c r="I17" s="92" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="18" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B18" s="63">
@@ -4148,8 +4187,12 @@
         <v>139</v>
       </c>
       <c r="G18" s="58"/>
-      <c r="H18" s="58"/>
-      <c r="I18" s="58"/>
+      <c r="H18" s="94">
+        <v>46327</v>
+      </c>
+      <c r="I18" s="92" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="19" spans="2:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B19" s="63">
@@ -4168,8 +4211,12 @@
         <v>141</v>
       </c>
       <c r="G19" s="61"/>
-      <c r="H19" s="61"/>
-      <c r="I19" s="61"/>
+      <c r="H19" s="94">
+        <v>46357</v>
+      </c>
+      <c r="I19" s="93" t="s">
+        <v>141</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4246,16 +4293,16 @@
       <c r="I3" s="63" t="s">
         <v>325</v>
       </c>
-      <c r="J3" s="90" t="s">
+      <c r="J3" s="88" t="s">
         <v>322</v>
       </c>
-      <c r="K3" s="90" t="s">
+      <c r="K3" s="88" t="s">
         <v>323</v>
       </c>
-      <c r="L3" s="90" t="s">
+      <c r="L3" s="88" t="s">
         <v>324</v>
       </c>
-      <c r="M3" s="90" t="s">
+      <c r="M3" s="88" t="s">
         <v>326</v>
       </c>
       <c r="N3" s="63"/>
@@ -4456,16 +4503,16 @@
       <c r="I4" s="62">
         <v>1</v>
       </c>
-      <c r="J4" s="91">
+      <c r="J4" s="89">
         <v>1</v>
       </c>
-      <c r="K4" s="91">
+      <c r="K4" s="89">
         <v>1</v>
       </c>
-      <c r="L4" s="91">
+      <c r="L4" s="89">
         <v>1</v>
       </c>
-      <c r="M4" s="91">
+      <c r="M4" s="89">
         <v>1</v>
       </c>
     </row>
@@ -4489,16 +4536,16 @@
       <c r="I5" s="62">
         <v>0.92</v>
       </c>
-      <c r="J5" s="91">
+      <c r="J5" s="89">
         <v>0.92</v>
       </c>
-      <c r="K5" s="91">
+      <c r="K5" s="89">
         <v>0.89</v>
       </c>
-      <c r="L5" s="91">
+      <c r="L5" s="89">
         <v>0.6</v>
       </c>
-      <c r="M5" s="91">
+      <c r="M5" s="89">
         <v>0.56000000000000005</v>
       </c>
     </row>
@@ -4522,16 +4569,16 @@
       <c r="I6" s="62">
         <v>0.83</v>
       </c>
-      <c r="J6" s="91">
+      <c r="J6" s="89">
         <v>0.84</v>
       </c>
-      <c r="K6" s="91">
+      <c r="K6" s="89">
         <v>0.79</v>
       </c>
-      <c r="L6" s="91">
+      <c r="L6" s="89">
         <v>0.52</v>
       </c>
-      <c r="M6" s="91">
+      <c r="M6" s="89">
         <v>0.49</v>
       </c>
     </row>
@@ -4555,16 +4602,16 @@
       <c r="I7" s="62">
         <v>0.77</v>
       </c>
-      <c r="J7" s="91">
+      <c r="J7" s="89">
         <v>0.74</v>
       </c>
-      <c r="K7" s="91">
+      <c r="K7" s="89">
         <v>0.69</v>
       </c>
-      <c r="L7" s="91">
+      <c r="L7" s="89">
         <v>0.45</v>
       </c>
-      <c r="M7" s="91">
+      <c r="M7" s="89">
         <v>0.43</v>
       </c>
     </row>
@@ -4588,16 +4635,16 @@
       <c r="I8" s="62">
         <v>0.7</v>
       </c>
-      <c r="J8" s="91">
+      <c r="J8" s="89">
         <v>0.65</v>
       </c>
-      <c r="K8" s="91">
+      <c r="K8" s="89">
         <v>0.59</v>
       </c>
-      <c r="L8" s="91">
+      <c r="L8" s="89">
         <v>0.4</v>
       </c>
-      <c r="M8" s="91">
+      <c r="M8" s="89">
         <v>0.38</v>
       </c>
     </row>
@@ -4621,16 +4668,16 @@
       <c r="I9" s="62">
         <v>0.65</v>
       </c>
-      <c r="J9" s="91">
+      <c r="J9" s="89">
         <v>0.56999999999999995</v>
       </c>
-      <c r="K9" s="91">
+      <c r="K9" s="89">
         <v>0.52</v>
       </c>
-      <c r="L9" s="91">
+      <c r="L9" s="89">
         <v>0.37</v>
       </c>
-      <c r="M9" s="91">
+      <c r="M9" s="89">
         <v>0.35</v>
       </c>
     </row>
@@ -7400,26 +7447,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="90" t="s">
         <v>303</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="89" t="s">
+      <c r="A2" s="91" t="s">
         <v>304</v>
       </c>
-      <c r="B2" s="89"/>
-      <c r="C2" s="89"/>
-      <c r="D2" s="89"/>
-      <c r="E2" s="89"/>
-      <c r="F2" s="89"/>
-      <c r="G2" s="89"/>
+      <c r="B2" s="91"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="91"/>
     </row>
     <row r="3" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="71" t="s">
@@ -8015,18 +8062,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="90" t="s">
         <v>311</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="89" t="s">
+      <c r="A2" s="91" t="s">
         <v>312</v>
       </c>
-      <c r="B2" s="89"/>
-      <c r="C2" s="89"/>
+      <c r="B2" s="91"/>
+      <c r="C2" s="91"/>
     </row>
     <row r="3" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="71" t="s">
@@ -8091,20 +8138,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="88" t="s">
+      <c r="A1" s="90" t="s">
         <v>319</v>
       </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
+      <c r="B1" s="90"/>
+      <c r="C1" s="90"/>
+      <c r="D1" s="90"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="89" t="s">
+      <c r="A2" s="91" t="s">
         <v>320</v>
       </c>
-      <c r="B2" s="89"/>
-      <c r="C2" s="89"/>
-      <c r="D2" s="89"/>
+      <c r="B2" s="91"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
     </row>
     <row r="3" spans="1:4" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="71" t="s">

</xml_diff>

<commit_message>
feedbacks incorporated and bugs fixed
</commit_message>
<xml_diff>
--- a/NAP mock data.xlsx
+++ b/NAP mock data.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC561869-D2D5-4A1D-824E-BD4C11E46DD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00EC873D-5AD3-43D0-967E-2A55EC5A7505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Market growth" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="361" uniqueCount="327">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="323">
   <si>
     <t>Year</t>
   </si>
@@ -997,18 +997,6 @@
     <t>8.4 mo</t>
   </si>
   <si>
-    <t>Access</t>
-  </si>
-  <si>
-    <t>MMIT Formulary Coverage Data</t>
-  </si>
-  <si>
-    <t>Fulfilment</t>
-  </si>
-  <si>
-    <t>Improving</t>
-  </si>
-  <si>
     <t>Compliance</t>
   </si>
   <si>
@@ -1057,9 +1045,6 @@
     <t>Primary care</t>
   </si>
   <si>
-    <t>Lipid spec.</t>
-  </si>
-  <si>
     <t>Liphendra Compliance — monthly source data</t>
   </si>
   <si>
@@ -1082,6 +1067,9 @@
   </si>
   <si>
     <t>Leqvio</t>
+  </si>
+  <si>
+    <t>Other spec.</t>
   </si>
 </sst>
 </file>
@@ -1808,12 +1796,6 @@
     <xf numFmtId="9" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1822,6 +1804,12 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4067,10 +4055,10 @@
         <v>128</v>
       </c>
       <c r="G13" s="52"/>
-      <c r="H13" s="93" t="s">
+      <c r="H13" s="91" t="s">
         <v>58</v>
       </c>
-      <c r="I13" s="93" t="s">
+      <c r="I13" s="91" t="s">
         <v>128</v>
       </c>
     </row>
@@ -4091,10 +4079,10 @@
         <v>131</v>
       </c>
       <c r="G14" s="58"/>
-      <c r="H14" s="94">
+      <c r="H14" s="92">
         <v>46204</v>
       </c>
-      <c r="I14" s="92" t="s">
+      <c r="I14" s="90" t="s">
         <v>131</v>
       </c>
     </row>
@@ -4115,10 +4103,10 @@
         <v>133</v>
       </c>
       <c r="G15" s="58"/>
-      <c r="H15" s="94">
+      <c r="H15" s="92">
         <v>46235</v>
       </c>
-      <c r="I15" s="92" t="s">
+      <c r="I15" s="90" t="s">
         <v>133</v>
       </c>
     </row>
@@ -4139,10 +4127,10 @@
         <v>135</v>
       </c>
       <c r="G16" s="58"/>
-      <c r="H16" s="94">
+      <c r="H16" s="92">
         <v>46266</v>
       </c>
-      <c r="I16" s="92" t="s">
+      <c r="I16" s="90" t="s">
         <v>135</v>
       </c>
     </row>
@@ -4163,10 +4151,10 @@
         <v>137</v>
       </c>
       <c r="G17" s="58"/>
-      <c r="H17" s="94">
+      <c r="H17" s="92">
         <v>46296</v>
       </c>
-      <c r="I17" s="92" t="s">
+      <c r="I17" s="90" t="s">
         <v>137</v>
       </c>
     </row>
@@ -4187,10 +4175,10 @@
         <v>139</v>
       </c>
       <c r="G18" s="58"/>
-      <c r="H18" s="94">
+      <c r="H18" s="92">
         <v>46327</v>
       </c>
-      <c r="I18" s="92" t="s">
+      <c r="I18" s="90" t="s">
         <v>139</v>
       </c>
     </row>
@@ -4211,10 +4199,10 @@
         <v>141</v>
       </c>
       <c r="G19" s="61"/>
-      <c r="H19" s="94">
+      <c r="H19" s="92">
         <v>46357</v>
       </c>
-      <c r="I19" s="93" t="s">
+      <c r="I19" s="91" t="s">
         <v>141</v>
       </c>
     </row>
@@ -4291,19 +4279,19 @@
         <v>146</v>
       </c>
       <c r="I3" s="63" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="J3" s="88" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="K3" s="88" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="L3" s="88" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="M3" s="88" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="N3" s="63"/>
       <c r="O3" s="63"/>
@@ -7362,75 +7350,38 @@
         <v>292</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B8" s="67" t="s">
         <v>298</v>
       </c>
       <c r="C8" s="54">
-        <v>0.41</v>
-      </c>
-      <c r="D8" s="54">
-        <v>0.35</v>
-      </c>
-      <c r="E8" s="54">
-        <v>0.38</v>
-      </c>
-      <c r="F8" s="55">
-        <v>0.39</v>
+        <v>0.84</v>
+      </c>
+      <c r="D8" s="67" t="s">
+        <v>130</v>
+      </c>
+      <c r="E8" s="67" t="s">
+        <v>130</v>
+      </c>
+      <c r="F8" s="54">
+        <v>0.83</v>
       </c>
       <c r="G8" s="67" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="H8" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="67" t="s">
-        <v>300</v>
-      </c>
-      <c r="C9" s="54">
-        <v>0.9</v>
-      </c>
-      <c r="D9" s="54">
-        <v>0.82</v>
-      </c>
-      <c r="E9" s="54">
-        <v>0.85</v>
-      </c>
-      <c r="F9" s="55">
-        <v>0.87</v>
-      </c>
-      <c r="G9" s="67" t="s">
-        <v>301</v>
-      </c>
-      <c r="H9" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="10" spans="2:8" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="67" t="s">
-        <v>302</v>
-      </c>
-      <c r="C10" s="54">
-        <v>0.84</v>
-      </c>
-      <c r="D10" s="67" t="s">
-        <v>130</v>
-      </c>
-      <c r="E10" s="67" t="s">
-        <v>130</v>
-      </c>
-      <c r="F10" s="54">
-        <v>0.83</v>
-      </c>
-      <c r="G10" s="67" t="s">
-        <v>294</v>
-      </c>
-      <c r="H10" t="s">
-        <v>292</v>
-      </c>
-    </row>
+      <c r="B9" s="67"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="54"/>
+      <c r="E9" s="54"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="67"/>
+    </row>
+    <row r="10" spans="2:8" ht="22.95" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7447,48 +7398,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="90" t="s">
-        <v>303</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
+      <c r="A1" s="93" t="s">
+        <v>299</v>
+      </c>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
+      <c r="E1" s="93"/>
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="91" t="s">
-        <v>304</v>
-      </c>
-      <c r="B2" s="91"/>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
-      <c r="E2" s="91"/>
-      <c r="F2" s="91"/>
-      <c r="G2" s="91"/>
+      <c r="A2" s="94" t="s">
+        <v>300</v>
+      </c>
+      <c r="B2" s="94"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="94"/>
     </row>
     <row r="3" spans="1:7" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="71" t="s">
         <v>58</v>
       </c>
       <c r="B3" s="71" t="s">
+        <v>301</v>
+      </c>
+      <c r="C3" s="71" t="s">
+        <v>302</v>
+      </c>
+      <c r="D3" s="71" t="s">
+        <v>303</v>
+      </c>
+      <c r="E3" s="71" t="s">
+        <v>304</v>
+      </c>
+      <c r="F3" s="71" t="s">
         <v>305</v>
       </c>
-      <c r="C3" s="71" t="s">
+      <c r="G3" s="71" t="s">
         <v>306</v>
-      </c>
-      <c r="D3" s="71" t="s">
-        <v>307</v>
-      </c>
-      <c r="E3" s="71" t="s">
-        <v>308</v>
-      </c>
-      <c r="F3" s="71" t="s">
-        <v>309</v>
-      </c>
-      <c r="G3" s="71" t="s">
-        <v>310</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8062,61 +8013,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="90" t="s">
-        <v>311</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
+      <c r="A1" s="93" t="s">
+        <v>307</v>
+      </c>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="91" t="s">
-        <v>312</v>
-      </c>
-      <c r="B2" s="91"/>
-      <c r="C2" s="91"/>
+      <c r="A2" s="94" t="s">
+        <v>308</v>
+      </c>
+      <c r="B2" s="94"/>
+      <c r="C2" s="94"/>
     </row>
     <row r="3" spans="1:3" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="71" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="B3" s="71" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="C3" s="71" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="75" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="B4" s="76">
         <v>3200</v>
       </c>
       <c r="C4" s="77">
-        <v>6.1</v>
+        <v>9.1999999999999993</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="75" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="B5" s="76">
         <v>2600</v>
       </c>
       <c r="C5" s="77">
-        <v>3.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="75" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="B6" s="76">
         <v>900</v>
       </c>
       <c r="C6" s="77">
-        <v>9.1999999999999993</v>
+        <v>3.4</v>
       </c>
     </row>
   </sheetData>
@@ -8138,20 +8089,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="90" t="s">
-        <v>319</v>
-      </c>
-      <c r="B1" s="90"/>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
+      <c r="A1" s="93" t="s">
+        <v>314</v>
+      </c>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="91" t="s">
-        <v>320</v>
-      </c>
-      <c r="B2" s="91"/>
-      <c r="C2" s="91"/>
-      <c r="D2" s="91"/>
+      <c r="A2" s="94" t="s">
+        <v>315</v>
+      </c>
+      <c r="B2" s="94"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
     </row>
     <row r="3" spans="1:4" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="71" t="s">
@@ -8172,13 +8123,13 @@
         <v>46204</v>
       </c>
       <c r="B4" s="78">
-        <v>0.72</v>
+        <v>0.8</v>
       </c>
       <c r="C4" s="78">
         <v>0.79</v>
       </c>
       <c r="D4" s="75" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8186,13 +8137,13 @@
         <v>46235</v>
       </c>
       <c r="B5" s="78">
-        <v>0.76</v>
+        <v>0.8</v>
       </c>
       <c r="C5" s="78">
         <v>0.8</v>
       </c>
       <c r="D5" s="75" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8200,13 +8151,13 @@
         <v>46266</v>
       </c>
       <c r="B6" s="78">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="C6" s="78">
         <v>0.81</v>
       </c>
       <c r="D6" s="75" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8214,13 +8165,13 @@
         <v>46296</v>
       </c>
       <c r="B7" s="78">
-        <v>0.81</v>
+        <v>0.8</v>
       </c>
       <c r="C7" s="78">
         <v>0.82</v>
       </c>
       <c r="D7" s="75" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8228,13 +8179,13 @@
         <v>46327</v>
       </c>
       <c r="B8" s="78">
-        <v>0.83</v>
+        <v>0.8</v>
       </c>
       <c r="C8" s="78">
         <v>0.82</v>
       </c>
       <c r="D8" s="75" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -8242,13 +8193,13 @@
         <v>46357</v>
       </c>
       <c r="B9" s="78">
-        <v>0.84</v>
+        <v>0.8</v>
       </c>
       <c r="C9" s="78">
         <v>0.83</v>
       </c>
       <c r="D9" s="75" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>